<commit_message>
updated rule yaml and test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000004/positive/01/data/unit-test-coreid-CG0101-positive.xlsx
+++ b/rules/CORE-000004/positive/01/data/unit-test-coreid-CG0101-positive.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silvia.Faini\CORE\Rule_Authoring\core-contributor\rules\CORE-000004\positive\01\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\CORE-000004\positive\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DDB934-DA7A-4D91-8BC0-16D602FD4709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBB02D0-28D7-42F8-8101-08A9B84365B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -286,15 +286,18 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -667,9 +670,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -677,7 +680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -696,9 +699,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -706,7 +709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -725,9 +728,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:T20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -789,7 +795,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
@@ -851,7 +857,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>48</v>
       </c>
@@ -913,7 +919,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>12</v>
       </c>
@@ -975,7 +981,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>50</v>
       </c>
@@ -1037,7 +1043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>50</v>
       </c>
@@ -1099,7 +1105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>50</v>
       </c>
@@ -1161,7 +1167,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>50</v>
       </c>
@@ -1223,7 +1229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>50</v>
       </c>
@@ -1285,7 +1291,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>50</v>
       </c>
@@ -1305,7 +1311,7 @@
         <v>54</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="H10" s="3">
         <v>5</v>
@@ -1347,7 +1353,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>50</v>
       </c>
@@ -1409,7 +1415,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>50</v>
       </c>
@@ -1471,7 +1477,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>50</v>
       </c>
@@ -1533,7 +1539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>50</v>
       </c>
@@ -1595,7 +1601,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>50</v>
       </c>
@@ -1657,7 +1663,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>50</v>
       </c>
@@ -1719,7 +1725,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>50</v>
       </c>
@@ -1781,7 +1787,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>50</v>
       </c>
@@ -1843,7 +1849,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>50</v>
       </c>
@@ -1905,7 +1911,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>50</v>
       </c>
@@ -1970,7 +1976,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:T11 A14:T20 A12:D12 F12:G12 I12:T12 A13:G13 I13:T13" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:T9 A14:T20 A12:D12 F12:G12 I12:T12 A13:G13 I13:T13 A11:T11 A10:F10 H10:T10" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>